<commit_message>
v0.9.9.9: migrate MAME sample fixtures and locale from IspS to EGFP
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,26 +475,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>232</v>
+        <v>65</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CAG</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>GCG</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>233</v>
+        <v>66</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -544,12 +544,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>GCC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -575,31 +575,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>203</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>T</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GCG</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CCG</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -625,31 +625,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GAA</t>
+          <t>TTC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>CTC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -675,31 +675,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150</v>
+        <v>206</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>K</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CTG</t>
+          <t>GCA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GTG</t>
+          <t>AAG</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -725,31 +725,31 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GCG</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CCG</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>G6</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>combo</t>
+          <t>single</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -771,45 +771,45 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M007</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GAA</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>TGG</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PS_006</t>
+          <t>PS_007</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>combo</t>
+          <t>single</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -821,48 +821,148 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>M008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>203</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ACA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TTC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PS_008</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>M009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>99</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TTC</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AGC</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G9</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PS_009</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>WT</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B11" t="n">
         <v>0</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>wt</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>control</t>
         </is>

</xml_diff>

<commit_message>
chore(samples): regenerate the MAME sample set so step 4 builds from it
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="expected_mutations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="expected_mutations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,30 +471,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>Y67H</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -521,30 +521,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M002</t>
+          <t>F100S</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>TTC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -571,30 +571,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M003</t>
+          <t>S148P</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>203</v>
+        <v>148</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -621,30 +621,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M004</t>
+          <t>H149D</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64</v>
+        <v>149</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CTC</t>
+          <t>GAC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -671,30 +671,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M005</t>
+          <t>M154T</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GCA</t>
+          <t>ATG</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AAG</t>
+          <t>ACG</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -721,15 +721,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>V164A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>65</v>
+        <v>164</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>GTG</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GCC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -771,30 +771,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>I168T</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>66</v>
+        <v>168</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>ATC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TGG</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -821,11 +821,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>T204Y</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -834,17 +834,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -871,30 +871,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>S206T</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>99</v>
+        <v>206</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -921,48 +921,100 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>A207K</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>207</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>AAG</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PS_010</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>WT</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>wt</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>control</t>
         </is>

</xml_diff>

<commit_message>
v0.16.40: sample data that finishes the step 4 build it starts
Regenerate the bundled MAME sample set from one generator so step 4 builds from it, without bundling a nanopore run. Adds the Analyze verdict workbook, raw-scale and variant-labeled long formats, and a numeric-ID confirmation report; the results screen now reads the pipeline-produced fixture.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="expected_mutations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="expected_mutations" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,30 +471,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>Y67H</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>H</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -521,30 +521,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M002</t>
+          <t>F100S</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>TTC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -571,30 +571,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M003</t>
+          <t>S148P</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>203</v>
+        <v>148</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>P</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -621,30 +621,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M004</t>
+          <t>H149D</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64</v>
+        <v>149</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CTC</t>
+          <t>GAC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -671,30 +671,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M005</t>
+          <t>M154T</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GCA</t>
+          <t>ATG</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AAG</t>
+          <t>ACG</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -721,15 +721,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>V164A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>65</v>
+        <v>164</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>GTG</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GCC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -771,30 +771,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>I168T</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>66</v>
+        <v>168</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>ATC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TGG</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -821,11 +821,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>T204Y</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -834,17 +834,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>TAC</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -871,30 +871,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>S206T</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>99</v>
+        <v>206</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>TCC</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>ACC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -921,48 +921,100 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>A207K</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>207</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>AAG</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PS_010</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>WT</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>wt</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>control</t>
         </is>

</xml_diff>

<commit_message>
chore(samples): derive the MAME plate from the KURO prediction so the demo is one campaign
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -471,30 +471,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Y67H</t>
+          <t>F28A</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>TTC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -521,30 +521,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F100S</t>
+          <t>H78A</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -571,30 +571,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S148P</t>
+          <t>A88V</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>V</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>GTC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -621,30 +621,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H149D</t>
+          <t>R97A</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>149</v>
+        <v>97</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>R</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>CGC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GAC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -671,30 +671,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M154T</t>
+          <t>I124A</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ATG</t>
+          <t>ATC</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ACG</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -721,15 +721,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>V164A</t>
+          <t>N150A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GTG</t>
+          <t>AAC</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GCG</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -771,30 +771,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>I168T</t>
+          <t>K163A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ATC</t>
+          <t>AAG</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -821,30 +821,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T204Y</t>
+          <t>G175A</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>204</v>
+        <v>175</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GGC</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -871,30 +871,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S206T</t>
+          <t>G190A</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>GGC</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -921,30 +921,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A207K</t>
+          <t>H200A</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>GCC</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>AAG</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
v0.16.41: one campaign, from the prediction to the plate
Derive the MAME plate from the bundled KURO EVOLVEpro prediction by running the primer design, so the two halves of the sample data describe one experiment. Adds a chain test that reads the shipped files and fails when they diverge.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -471,30 +471,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Y67H</t>
+          <t>F28A</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>TTC</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -521,30 +521,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F100S</t>
+          <t>H78A</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>TTC</t>
+          <t>CAC</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -571,30 +571,30 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S148P</t>
+          <t>A88V</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>148</v>
+        <v>88</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>V</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AGC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>GTC</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -621,30 +621,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H149D</t>
+          <t>R97A</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>149</v>
+        <v>97</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>R</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>CGC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>GAC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -671,30 +671,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M154T</t>
+          <t>I124A</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ATG</t>
+          <t>ATC</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ACG</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -721,15 +721,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>V164A</t>
+          <t>N150A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -739,12 +739,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GTG</t>
+          <t>AAC</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>GCG</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -771,30 +771,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>I168T</t>
+          <t>K163A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ATC</t>
+          <t>AAG</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -821,30 +821,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T204Y</t>
+          <t>G175A</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>204</v>
+        <v>175</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GGC</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>GCG</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -871,30 +871,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S206T</t>
+          <t>G190A</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TCC</t>
+          <t>GGC</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>GCC</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -921,30 +921,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A207K</t>
+          <t>H200A</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>GCC</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>AAG</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>

<commit_message>
v0.16.42: three barcodes, and every verdict the pipeline can reach
Triplicate the bundled MAME sample across NB01-NB03, surface all eight verdict classes on the selected replicate, and seed sample file paths into every step. See CHANGELOG for detail.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
+++ b/src-tauri/samples/mame/03_mame_expected_mutations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -971,50 +971,350 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Q205A</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>205</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CAG</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>GCG</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PS_011</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>K210A</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>210</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>GCA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PS_012</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>K215A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>215</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AAG</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>GCG</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PS_013</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A227V</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>227</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>GTC</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PS_014</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D235A</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>235</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GAC</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PS_015</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>K239A</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>239</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>AAG</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>GCG</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>PS_016</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>designed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>WT</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>G0</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>wt</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>control</t>
         </is>

</xml_diff>